<commit_message>
Update candidate details with real name, email, ID, and repo URL
</commit_message>
<xml_diff>
--- a/output/IncuBrix_Submission.xlsx
+++ b/output/IncuBrix_Submission.xlsx
@@ -1037,7 +1037,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>SASTRA-2027-GROWTH</t>
+          <t>227004127@sastra.ac.in</t>
         </is>
       </c>
       <c r="D13" s="1" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>YOUR NAME</t>
+          <t>Venkatvishaal Thalamudupula Srinivaas</t>
         </is>
       </c>
       <c r="D14" s="16" t="n">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>your@email.com</t>
+          <t>venkatvishaalts@gmail.com</t>
         </is>
       </c>
       <c r="D15" s="18" t="n">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>2026-09-04 19:07</t>
+          <t>2026-09-05 20:02</t>
         </is>
       </c>
       <c r="D17" s="18" t="n">
@@ -1162,7 +1162,11 @@
           <t>AI/tools used</t>
         </is>
       </c>
-      <c r="B18" s="14" t="n"/>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Google Gemini (Antigravity IDE) — code generation and architecture; YouTube Data API v3 — primary data source. All logic, qualification criteria, and evidence reviewed manually.</t>
+        </is>
+      </c>
       <c r="D18" s="20" t="n">
         <v>5</v>
       </c>
@@ -1185,7 +1189,7 @@
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>https://github.com/youruser/incubrix-lead-engine</t>
+          <t>https://github.com/venkatvishaal/GROWTH_INCUBRIX</t>
         </is>
       </c>
     </row>
@@ -1212,11 +1216,7 @@
           <t>Technical demo URL</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="B21" s="14" t="inlineStr"/>
       <c r="D21" s="76" t="n"/>
       <c r="H21" s="77" t="n"/>
     </row>

</xml_diff>

<commit_message>
Update AI/tools used field to 'Antigravity used for automation'
</commit_message>
<xml_diff>
--- a/output/IncuBrix_Submission.xlsx
+++ b/output/IncuBrix_Submission.xlsx
@@ -1139,7 +1139,7 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>2026-09-05 20:02</t>
+          <t>2026-09-05 20:06</t>
         </is>
       </c>
       <c r="D17" s="18" t="n">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Google Gemini (Antigravity IDE) — code generation and architecture; YouTube Data API v3 — primary data source. All logic, qualification criteria, and evidence reviewed manually.</t>
+          <t>Antigravity used for automation</t>
         </is>
       </c>
       <c r="D18" s="20" t="n">

</xml_diff>